<commit_message>
Sulfur aquatic tox, updates
- add some species/terms
- unify "measured" column

Our current column definition for "measured" for the aquatic toxicity
table (should be integrated in the package somewhere).

"nom" for nominal concentrations,
"amm" for arithmetic mean measured concentrations,
"gmm" for geometric mean measured concentrations,
"mm" for mean measured concentrations,
"im" for initial measured oder initial mean measured concentration,
"fm" for final measured,
"twa" for time-weighted average measured ,
“sol” stands for “solubility-limited”, indicating that the value was not experimentally measured but that the solubility limit was used instead
</commit_message>
<xml_diff>
--- a/data_generation/10_aquatic_toxicity/ametoctradin_aquatic_toxicity.xlsx
+++ b/data_generation/10_aquatic_toxicity/ametoctradin_aquatic_toxicity.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\aquatic_toxicity\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="O:\Data-Work\41_AssessmentPPP-RE\412.34_Projekte\054_derappp\05_Daten\Input\10_aquatic_toxicity\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC720E9F-F3C1-4483-B68C-531E87CD7533}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED884664-8D14-408D-BE4D-918345A7FE6C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19080" yWindow="-2850" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aquatic toxicity" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aquatic toxicity'!$A$1:$V$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Aquatic toxicity'!$A$1:$V$18</definedName>
   </definedNames>
   <calcPr calcId="0"/>
   <extLst>
@@ -189,9 +189,6 @@
     <t>28 d</t>
   </si>
   <si>
-    <t>mg a.s./kg sediment</t>
-  </si>
-  <si>
     <t>biomass</t>
   </si>
   <si>
@@ -220,6 +217,9 @@
   </si>
   <si>
     <t>Sediment endpoint currently not used</t>
+  </si>
+  <si>
+    <t>mg/kg</t>
   </si>
 </sst>
 </file>
@@ -663,7 +663,7 @@
     </row>
     <row r="2" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C2" t="s">
         <v>22</v>
@@ -708,18 +708,18 @@
         <v>25</v>
       </c>
       <c r="T2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="U2" t="s">
         <v>50</v>
       </c>
       <c r="V2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="3" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C3" t="s">
         <v>28</v>
@@ -767,12 +767,12 @@
         <v>50</v>
       </c>
       <c r="V3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
         <v>29</v>
@@ -820,12 +820,12 @@
         <v>50</v>
       </c>
       <c r="V4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="5" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C5" t="s">
         <v>30</v>
@@ -873,15 +873,15 @@
         <v>50</v>
       </c>
       <c r="V5" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C6" t="s">
         <v>22</v>
@@ -929,15 +929,15 @@
         <v>50</v>
       </c>
       <c r="V6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C7" t="s">
         <v>22</v>
@@ -973,24 +973,24 @@
         <v>67</v>
       </c>
       <c r="R7" t="s">
+        <v>60</v>
+      </c>
+      <c r="S7" t="s">
         <v>61</v>
       </c>
-      <c r="S7" t="s">
-        <v>62</v>
-      </c>
       <c r="T7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="U7" t="s">
         <v>50</v>
       </c>
       <c r="V7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="8" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C8" t="s">
         <v>31</v>
@@ -1038,12 +1038,12 @@
         <v>50</v>
       </c>
       <c r="V8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
         <v>31</v>
@@ -1088,15 +1088,15 @@
         <v>50</v>
       </c>
       <c r="V9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C10" t="s">
         <v>31</v>
@@ -1144,15 +1144,15 @@
         <v>50</v>
       </c>
       <c r="V10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
@@ -1191,27 +1191,27 @@
         <v>68</v>
       </c>
       <c r="R11" t="s">
+        <v>60</v>
+      </c>
+      <c r="S11" t="s">
         <v>61</v>
       </c>
-      <c r="S11" t="s">
-        <v>62</v>
-      </c>
       <c r="T11" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="U11" t="s">
         <v>50</v>
       </c>
       <c r="V11" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
         <v>51</v>
@@ -1232,7 +1232,7 @@
         <v>221.56</v>
       </c>
       <c r="N12" t="s">
-        <v>53</v>
+        <v>63</v>
       </c>
       <c r="P12" t="s">
         <v>49</v>
@@ -1241,21 +1241,21 @@
         <v>68</v>
       </c>
       <c r="R12" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="S12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="U12" t="s">
         <v>50</v>
       </c>
       <c r="V12" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C13" t="s">
         <v>33</v>
@@ -1270,7 +1270,7 @@
         <v>45</v>
       </c>
       <c r="I13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K13" t="s">
         <v>32</v>
@@ -1303,12 +1303,12 @@
         <v>50</v>
       </c>
       <c r="V13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C14" t="s">
         <v>33</v>
@@ -1356,15 +1356,15 @@
         <v>50</v>
       </c>
       <c r="V14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C15" t="s">
         <v>33</v>
@@ -1379,7 +1379,7 @@
         <v>45</v>
       </c>
       <c r="I15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K15" t="s">
         <v>32</v>
@@ -1412,15 +1412,15 @@
         <v>50</v>
       </c>
       <c r="V15" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
         <v>33</v>
@@ -1468,15 +1468,15 @@
         <v>50</v>
       </c>
       <c r="V16" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C17" t="s">
         <v>33</v>
@@ -1491,7 +1491,7 @@
         <v>45</v>
       </c>
       <c r="I17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="K17" t="s">
         <v>32</v>
@@ -1512,27 +1512,27 @@
         <v>68</v>
       </c>
       <c r="R17" t="s">
+        <v>60</v>
+      </c>
+      <c r="S17" t="s">
         <v>61</v>
       </c>
-      <c r="S17" t="s">
-        <v>62</v>
-      </c>
       <c r="T17" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="U17" t="s">
         <v>50</v>
       </c>
       <c r="V17" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="18" spans="1:22" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C18" t="s">
         <v>33</v>
@@ -1568,23 +1568,23 @@
         <v>68</v>
       </c>
       <c r="R18" t="s">
+        <v>60</v>
+      </c>
+      <c r="S18" t="s">
         <v>61</v>
       </c>
-      <c r="S18" t="s">
-        <v>62</v>
-      </c>
       <c r="T18" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="U18" t="s">
         <v>50</v>
       </c>
       <c r="V18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V35" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:V18" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>

</xml_diff>